<commit_message>
Update affiliate product links under comments (120 fresh Shopee affiliate links across 6 categories)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/affiliate_data/สัตว์เลี้ยง.xlsx
+++ b/affiliate_data/สัตว์เลี้ยง.xlsx
@@ -445,10 +445,10 @@
         <v>ยกโหล Nekko อาหารเปียกแมว 70 กรัม12ซอง</v>
       </c>
       <c r="C2" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mofbqutr8kcu6a.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823r0-mp0pjfpweby84e.webp</v>
       </c>
       <c r="D2" t="str">
-        <v>159.00</v>
+        <v>158.00</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -457,7 +457,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>ขายได้ 26 ชิ้น</v>
+        <v>ขายได้ 5พัน+ ชิ้น</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -466,7 +466,7 @@
         <v>https://shopee.co.th/product/0/48910813131</v>
       </c>
       <c r="J2" t="str">
-        <v>https://s.shopee.co.th/1BJb9Qw4hN</v>
+        <v>https://s.shopee.co.th/7AayLy4TAu</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -480,37 +480,37 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>FABLEME —PET BASKET เข่งใส่แมว ตระกร้าที่นอนแมวแบบเข่ง สไตล์มินิมอลง</v>
+        <v>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</v>
       </c>
       <c r="C3" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztk-mnrcaodqhb0k02.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</v>
       </c>
       <c r="D3" t="str">
-        <v>220.00</v>
+        <v>7714.00</v>
       </c>
       <c r="E3" t="str">
         <v/>
       </c>
       <c r="F3" t="str">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G3" t="str">
-        <v>ขายได้ 7 ชิ้น</v>
+        <v>ขายได้ 1พัน+ ชิ้น</v>
       </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>https://shopee.co.th/product/0/44859868817</v>
+        <v>https://shopee.co.th/product/0/25001294340</v>
       </c>
       <c r="J3" t="str">
-        <v>https://s.shopee.co.th/3B4fX6y9c8</v>
+        <v>https://s.shopee.co.th/5L9KAbNLFq</v>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -518,37 +518,37 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</v>
+        <v>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</v>
       </c>
       <c r="C4" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztm-mp1zyxmcgm4r44.webp</v>
       </c>
       <c r="D4" t="str">
-        <v>210.00</v>
+        <v>9990.00</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="G4" t="str">
-        <v>ขายได้ 2พัน+ ชิ้น</v>
+        <v>ขายได้ 623 ชิ้น</v>
       </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>https://shopee.co.th/product/0/25456988939</v>
+        <v>https://shopee.co.th/product/0/24369249453</v>
       </c>
       <c r="J4" t="str">
-        <v>https://s.shopee.co.th/4AxCiwxzUR</v>
+        <v>https://s.shopee.co.th/2qRzC0bKNG</v>
       </c>
       <c r="K4" t="str">
         <v/>
       </c>
       <c r="L4" t="str">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -556,37 +556,37 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>4-6L เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ รองรับWiFi &amp; APP เครื่องให้อาหาร เครื่องให้อาหารแมวอัตโนมัติ สําหรับสัตว์เลี้ยง</v>
+        <v>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม</v>
       </c>
       <c r="C5" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mmmvfucpjm6db4.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</v>
       </c>
       <c r="D5" t="str">
-        <v>491.00</v>
+        <v>1999.00</v>
       </c>
       <c r="E5" t="str">
         <v/>
       </c>
       <c r="F5" t="str">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="G5" t="str">
-        <v>ขายได้ 229 ชิ้น</v>
+        <v>ขายได้ 1พัน+ ชิ้น</v>
       </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>https://shopee.co.th/product/0/27544329163</v>
+        <v>https://shopee.co.th/product/0/22675992236</v>
       </c>
       <c r="J5" t="str">
-        <v>https://s.shopee.co.th/7KuEUluFn0</v>
+        <v>https://s.shopee.co.th/AAEZvUHexi</v>
       </c>
       <c r="K5" t="str">
         <v/>
       </c>
       <c r="L5" t="str">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         <v>https://down-bs-th.img.susercontent.com/th-11134207-81zto-mopbxox2cfm73f.webp</v>
       </c>
       <c r="D6" t="str">
-        <v>542.00</v>
+        <v>547.00</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -618,7 +618,7 @@
         <v>https://shopee.co.th/product/0/20348607344</v>
       </c>
       <c r="J6" t="str">
-        <v>https://s.shopee.co.th/2BC8LHMRmu</v>
+        <v>https://s.shopee.co.th/4AxMmSnMyM</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -632,37 +632,37 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</v>
+        <v>[🔥ใส่โค้ดลดเพิ่ม] Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK V.3 และ CATLINK V.3 Ultra</v>
       </c>
       <c r="C7" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0k-mbdr25xh8y299a.webp</v>
       </c>
       <c r="D7" t="str">
-        <v>5212.00</v>
+        <v>13900.00</v>
       </c>
       <c r="E7" t="str">
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="G7" t="str">
-        <v>ขายได้ 961 ชิ้น</v>
+        <v>ขายได้ 4พัน+ ชิ้น</v>
       </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>https://shopee.co.th/product/0/26274333150</v>
+        <v>https://shopee.co.th/product/0/5507071097</v>
       </c>
       <c r="J7" t="str">
-        <v>https://s.shopee.co.th/3LO5jQQjkG</v>
+        <v>https://s.shopee.co.th/5fmAZDqFhJ</v>
       </c>
       <c r="K7" t="str">
         <v/>
       </c>
       <c r="L7" t="str">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -670,37 +670,37 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>HYKI - NOTTY Global Version - ห้องน้ำแมวอัตโนมัติ NOTTY by HYKI</v>
+        <v>[ประกันศูนย์ไทย] Oneisall Pet Grooming Vacuum Kit 8 in 1 ตัดขนแมว เครื่องดูดขนแมว ไดร์เป่าขนสุนัข ขนาด2.5L รุ่น BM1</v>
       </c>
       <c r="C8" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m4frb6n3mu1683.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0h-mdtub2gcu0oe50.webp</v>
       </c>
       <c r="D8" t="str">
-        <v>7888.00</v>
+        <v>5372.00</v>
       </c>
       <c r="E8" t="str">
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 963 ชิ้น</v>
       </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>https://shopee.co.th/product/0/25001294340</v>
+        <v>https://shopee.co.th/product/0/26274333150</v>
       </c>
       <c r="J8" t="str">
-        <v>https://s.shopee.co.th/qgkkpnnSC</v>
+        <v>https://s.shopee.co.th/3qKWNr61yu</v>
       </c>
       <c r="K8" t="str">
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -708,37 +708,37 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Rojeco เครื่องให้อาหารแมวอัตโนมัติ ปุ่มกด WIFI ควบคุมอัจฉริยะ ขนาด 2 ลิตร</v>
+        <v>Petology คอนโดแมวคุณภาพสูง แข็งแรง ทนทาน ใช้งานได้นาน รุ่น CD-01</v>
       </c>
       <c r="C9" t="str">
-        <v>https://down-bs-th.img.susercontent.com/cn-11134207-820l4-mlbsygs3nf9f31.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0i-mbdqw6sm2nna5d.webp</v>
       </c>
       <c r="D9" t="str">
-        <v>1363.00</v>
+        <v>11000.00</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>50</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 151 ชิ้น</v>
       </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>https://shopee.co.th/product/0/17998285056</v>
+        <v>https://shopee.co.th/product/0/6331670112</v>
       </c>
       <c r="J9" t="str">
-        <v>https://s.shopee.co.th/4AxCixh5W9</v>
+        <v>https://s.shopee.co.th/40dwaAECCx</v>
       </c>
       <c r="K9" t="str">
         <v/>
       </c>
       <c r="L9" t="str">
-        <v>11.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -746,37 +746,37 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>((12ซอง คละรสได้)) Pramy พรามี่ อาหารเปียกแมว หลากหลายรส ขนาด 70g. สูตรลูกแมว แมวโต แมวสูงวัย</v>
+        <v>[เลือกรสชาติได้] Purina ONE อาหารแมว 10 kg</v>
       </c>
       <c r="C10" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztd-mob33vjgv0gee0.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823ok-mp3h99k9jb4c65.webp</v>
       </c>
       <c r="D10" t="str">
-        <v>265.00</v>
+        <v>1499.00</v>
       </c>
       <c r="E10" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>16</v>
       </c>
       <c r="G10" t="str">
-        <v>ขายได้ 20 ชิ้น</v>
+        <v>ขายได้ 10พัน+ ชิ้น</v>
       </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>https://shopee.co.th/product/0/42978681219</v>
+        <v>https://shopee.co.th/product/0/42922380987</v>
       </c>
       <c r="J10" t="str">
-        <v>https://s.shopee.co.th/8KmlgcYJ3j</v>
+        <v>https://s.shopee.co.th/8ATVXp85zW</v>
       </c>
       <c r="K10" t="str">
         <v/>
       </c>
       <c r="L10" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -784,37 +784,37 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>PANDO Pet Dryer Room PD65 แพนโด้ เครื่องเป่าขน สำหรับสัตว์เลี้ยง รุ่น PD65 ตู้เป่าขน อัตโนม</v>
+        <v>BIO น้ำยาดับกลิ่น กลิ่นฉี่ กลิ่นมูลสัตว์เลี้ยง ล้างพื้นกลิ่นฉี่ ทำความสะอาด ปราศจากเชื้อโรค กลิ่นโอโซนบริสุทธิ์ 1,000 ml</v>
       </c>
       <c r="C11" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mojgkgp81dsf9b.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7r98x-lopnhfgn1k599e.webp</v>
       </c>
       <c r="D11" t="str">
-        <v>9990.00</v>
+        <v>209.00</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>41</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>ขายได้ 620 ชิ้น</v>
+        <v>ขายได้ 5พัน+ ชิ้น</v>
       </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>https://shopee.co.th/product/0/24369249453</v>
+        <v>https://shopee.co.th/product/0/25452334947</v>
       </c>
       <c r="J11" t="str">
-        <v>https://s.shopee.co.th/6L1hIwoeQ7</v>
+        <v>https://s.shopee.co.th/8V6LwRFcsS</v>
       </c>
       <c r="K11" t="str">
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -822,37 +822,37 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>ห้องน้ำแมวอัจฉริยะ ห้องน้ําแมวอัตโนมัติสามารถเก็บอุจจาระได้โดยอัตโนมัติตามการขับถ่ายของแมว หลีกเลี่ยงกลิ่นแปลก ๆ และยับย</v>
+        <v>Dr.Zkin Pet Spray ผลิตภัณฑ์สำหรับสัตว์เลี้ยง บำรุงขน ดับกลิ่น เพิ่มความหอม</v>
       </c>
       <c r="C12" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mkf3obhghekg6a.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mhh7zikraarne4.webp</v>
       </c>
       <c r="D12" t="str">
-        <v>3199.00</v>
+        <v>210.00</v>
       </c>
       <c r="E12" t="str">
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G12" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 2พัน+ ชิ้น</v>
       </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>https://shopee.co.th/product/0/3932344413</v>
+        <v>https://shopee.co.th/product/0/25456988939</v>
       </c>
       <c r="J12" t="str">
-        <v>https://s.shopee.co.th/20si8zFjb6</v>
+        <v>https://s.shopee.co.th/70HY9gQhNc</v>
       </c>
       <c r="K12" t="str">
         <v/>
       </c>
       <c r="L12" t="str">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -860,37 +860,37 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>กล่องเดินทางสัตว์เลี้ยง กรงหิ้วแมว กรงเดินทาง กล่องใส่สัตว์เลี้ยง กรงเดินทาง กล่องใส่สัตว์เลี้ยง</v>
+        <v>บ้านน็อคดาวน์ สำเร็จรูป</v>
       </c>
       <c r="C13" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0g-mbm7xxs7he1kb4.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasj-m7wxzwgmmrgc2f.webp</v>
       </c>
       <c r="D13" t="str">
-        <v>973.00</v>
+        <v>150000.00</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>58</v>
+        <v/>
       </c>
       <c r="G13" t="str">
-        <v>ขายได้ 267 ชิ้น</v>
+        <v/>
       </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>https://shopee.co.th/product/0/28534027308</v>
+        <v>https://shopee.co.th/product/0/25993261993</v>
       </c>
       <c r="J13" t="str">
-        <v>https://s.shopee.co.th/BR3xcUYD6</v>
+        <v>https://s.shopee.co.th/30lPOKnQ4s</v>
       </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -898,37 +898,37 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Pramy in Gravy 70g อาหารเปียกแมว แมวโต เกรวี่ 12ซอง สำหรับแมว2เดือนขึ้นไป Petus Kingkaew</v>
+        <v>Prowild โปรไวลด์ ซีเล็คเต็ด อาหารสุนัขทุกสายพันธุ์/ทุกช่วงวัย ขนาด 15 kg</v>
       </c>
       <c r="C14" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztl-mornhzyf1w5qc6.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ra0m-mbg6gn8vi82g66.webp</v>
       </c>
       <c r="D14" t="str">
-        <v>256.00</v>
+        <v>1590.00</v>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>45</v>
+        <v/>
       </c>
       <c r="G14" t="str">
-        <v>ขายได้ 63 ชิ้น</v>
+        <v>ขายได้ 30พัน+ ชิ้น</v>
       </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>https://shopee.co.th/product/0/27333954378</v>
+        <v>https://shopee.co.th/product/0/3670154648</v>
       </c>
       <c r="J14" t="str">
-        <v>https://s.shopee.co.th/2BC8LIUqJB</v>
+        <v>https://s.shopee.co.th/9fIJKaWMHK</v>
       </c>
       <c r="K14" t="str">
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -936,37 +936,37 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>navipet Smart Pet Dryer (Thai Version) ตู้เป่า ขนสัตว์เลี้ยง 72ลิตร O ZONE ฆ่าเชื้อได้ ประกันศูนย์ไทย</v>
+        <v>Petology ห้องน้ำแมวอัตโนมัติ ดีไซน์ใหญ่ รองรับแมวหลายตัว CATLINK Lite</v>
       </c>
       <c r="C15" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztn-mnqj2jpnw45hd8.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7ras9-mauvmoz6b0omd5.webp</v>
       </c>
       <c r="D15" t="str">
-        <v>7900.00</v>
+        <v>8800.00</v>
       </c>
       <c r="E15" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>43</v>
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 2พัน+ ชิ้น</v>
       </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
-        <v>https://shopee.co.th/product/0/25608755070</v>
+        <v>https://shopee.co.th/product/0/8904141232</v>
       </c>
       <c r="J15" t="str">
-        <v>https://s.shopee.co.th/LkU9vkgr8</v>
+        <v>https://s.shopee.co.th/60P0xquu84</v>
       </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -974,37 +974,37 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>ห้องน้ำแมวใหญ่ SMART CAT LITTER BO</v>
+        <v>แมว ไดร์เป่าผม 62 /82L ของใช้แมว เครื่องเป่าขนแมว อาบน้ําแมว ตู้อบแมว ตั้งเวลาได้ ไดร์เป่าขนแมว</v>
       </c>
       <c r="C16" t="str">
-        <v>https://down-bs-th.img.susercontent.com/sg-11134201-822yl-mhwpnsjh6k1wff.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134201-7rasf-maxkg8lg2suo1b.webp</v>
       </c>
       <c r="D16" t="str">
-        <v>1000.00</v>
+        <v>2933.00</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>51</v>
       </c>
       <c r="G16" t="str">
-        <v>ขายได้ 2พัน+ ชิ้น</v>
+        <v>ขายได้ 193 ชิ้น</v>
       </c>
       <c r="H16" t="str">
         <v/>
       </c>
       <c r="I16" t="str">
-        <v>https://shopee.co.th/product/0/54702667383</v>
+        <v>https://shopee.co.th/product/0/29425138487</v>
       </c>
       <c r="J16" t="str">
-        <v>https://s.shopee.co.th/7VDeh6StVB</v>
+        <v>https://s.shopee.co.th/9fIJKasq1a</v>
       </c>
       <c r="K16" t="str">
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -1012,37 +1012,37 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>F&amp;G วิลล่าแมว Cat Villa บ้านแมว กรงแมว วิลล่าไม้เนื้อแข็งตู้แมว ตู้โชว์ไม้เนื้อแข็ง วิลล่าแมวขนาดใหญ จัดส่งภายใน24ชั่วโม</v>
+        <v>คอกกระบะฮันเตอร์(Hunter Cage)</v>
       </c>
       <c r="C17" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasm-m3ytl0pibu8a95.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7qul0-lfgefx1hi2su42.webp</v>
       </c>
       <c r="D17" t="str">
-        <v>1999.00</v>
+        <v>11715.00</v>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>58</v>
+        <v>6</v>
       </c>
       <c r="G17" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 343 ชิ้น</v>
       </c>
       <c r="H17" t="str">
         <v/>
       </c>
       <c r="I17" t="str">
-        <v>https://shopee.co.th/product/0/22675992236</v>
+        <v>https://shopee.co.th/product/0/20378259987</v>
       </c>
       <c r="J17" t="str">
-        <v>https://s.shopee.co.th/3qKMKMpn2h</v>
+        <v>https://s.shopee.co.th/gNUc3Zcns</v>
       </c>
       <c r="K17" t="str">
         <v/>
       </c>
       <c r="L17" t="str">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
@@ -1050,37 +1050,37 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>ขนมแมวเลีย Me-O มีโอ 11 รสชาติ คละรสได้ 11/20/25/36 ซอง | ขนมแมว อาหารแมวเลีย อาหารเสริมแมว</v>
+        <v>[เลือกรสชาติได้] Purina One อาหารแมว 6.6กก</v>
       </c>
       <c r="C18" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztg-mnyj1j3uxe6ad5.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/sg-11134201-823rm-mp2iqoc9yo7jc3.webp</v>
       </c>
       <c r="D18" t="str">
-        <v>109.00</v>
+        <v>1149.00</v>
       </c>
       <c r="E18" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>9</v>
       </c>
       <c r="G18" t="str">
-        <v>ขายได้ 1พัน+ ชิ้น</v>
+        <v>ขายได้ 40พัน+ ชิ้น</v>
       </c>
       <c r="H18" t="str">
         <v/>
       </c>
       <c r="I18" t="str">
-        <v>https://shopee.co.th/product/0/17598844146</v>
+        <v>https://shopee.co.th/product/0/10998396488</v>
       </c>
       <c r="J18" t="str">
-        <v>https://s.shopee.co.th/1gFrkO6YwY</v>
+        <v>https://s.shopee.co.th/2LVib7bsCQ</v>
       </c>
       <c r="K18" t="str">
         <v/>
       </c>
       <c r="L18" t="str">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1088,37 +1088,37 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>สเปรย์น้ำหอมระงับกลิ่น แบรนด์พราวพาว สูตรอ่อนโยน สารสกัดจากธรรมชาติ 3 กลิ่น หอมละมุนชื่นใจ</v>
+        <v>🐈🐱Neakasa M1 2024 ห้องน้ำแมวอัตโนมัติ I Smart Cat Litter I จัดการข้อมูลแมว 3 ตัว I แอปควบคุมระยะไกล🐈🐱</v>
       </c>
       <c r="C19" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasa-m2usz5kign3644.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7rasi-m6oxwve9ydkf40.webp</v>
       </c>
       <c r="D19" t="str">
-        <v>169.00</v>
+        <v>10499.00</v>
       </c>
       <c r="E19" t="str">
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="G19" t="str">
-        <v>ขายได้ 3พัน+ ชิ้น</v>
+        <v>ขายได้ 835 ชิ้น</v>
       </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>https://shopee.co.th/product/0/25488591523</v>
+        <v>https://shopee.co.th/product/0/27771402652</v>
       </c>
       <c r="J19" t="str">
-        <v>https://s.shopee.co.th/17dlKLdcu</v>
+        <v>https://s.shopee.co.th/8V6LwSP3Kc</v>
       </c>
       <c r="K19" t="str">
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -1126,37 +1126,37 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>【พร้อมส่ง】 EGGแผ่นรองฉี่สุนัข ซึมซับไดีดี ต่อต้านแบคทีเรีย แผ่นรองฉี่ ผ้ารองฉี่สุนัข แผ่นรองฉี่แมว แผ่นรองซับ ทรายแมวCOD</v>
+        <v>Petoya คอลลาเจนญี่ปุ่นบำรุงข้อและขน สำหรับสุนัขและแมว สูตร Joint Focus + DHA</v>
       </c>
       <c r="C20" t="str">
-        <v>https://down-bs-th.img.susercontent.com/th-11134207-7qul3-lgylrzka8duw84.webp</v>
+        <v>https://down-bs-th.img.susercontent.com/th-11134207-7r98s-lxa2x1xegij3c3.webp</v>
       </c>
       <c r="D20" t="str">
-        <v>84.00</v>
+        <v>490.00</v>
       </c>
       <c r="E20" t="str">
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>58</v>
+        <v/>
       </c>
       <c r="G20" t="str">
-        <v>ขายได้ 400พัน+ ชิ้น</v>
+        <v>ขายได้ 3พัน+ ชิ้น</v>
       </c>
       <c r="H20" t="str">
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>https://shopee.co.th/product/0/22411724898</v>
+        <v>https://shopee.co.th/product/0/18483804394</v>
       </c>
       <c r="J20" t="str">
-        <v>https://s.shopee.co.th/AAEPs0miQH</v>
+        <v>https://s.shopee.co.th/6py7xOYUW1</v>
       </c>
       <c r="K20" t="str">
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -1170,16 +1170,16 @@
         <v>https://down-bs-th.img.susercontent.com/th-11134207-81ztf-mkdbuy6rdgjr2e.webp</v>
       </c>
       <c r="D21" t="str">
-        <v>1224.00</v>
+        <v>1186.00</v>
       </c>
       <c r="E21" t="str">
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G21" t="str">
-        <v>ขายได้ 164 ชิ้น</v>
+        <v>ขายได้ 198 ชิ้น</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -1188,7 +1188,7 @@
         <v>https://shopee.co.th/product/0/51205882798</v>
       </c>
       <c r="J21" t="str">
-        <v>https://s.shopee.co.th/9Uyj4mysUr</v>
+        <v>https://s.shopee.co.th/8Kmvk9b1wJ</v>
       </c>
       <c r="K21" t="str">
         <v/>

</xml_diff>